<commit_message>
app flask: separação da aba 3 em sub-abas
</commit_message>
<xml_diff>
--- a/updates_weekly/new_issues.xlsx
+++ b/updates_weekly/new_issues.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bcpsec-my.sharepoint.com/personal/ibinfo_bcpsecurities_com/Documents/Documentos/Market Update Automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bcpsec-my.sharepoint.com/personal/ibinfo_bcpsecurities_com/Documents/Documentos/Market Update Automation/updates_weekly/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="41" documentId="8_{94004D96-580F-404F-B8DE-3B882EEF74BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FDB21CB-1208-46AA-BBFF-EB7C2173F4F2}"/>
@@ -510,7 +510,7 @@
     <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="str">
         <f>_xll.BSRCH("FI:New Issues Brazil - EB2","cols=1;rows=25")</f>
-        <v>#N/A Requesting Data...</v>
+        <v>id</v>
       </c>
       <c r="F1" s="1"/>
     </row>

</xml_diff>

<commit_message>
app flask: adicionando back-end do resto das funcinalidades e tabelas de holders e volume
</commit_message>
<xml_diff>
--- a/updates_weekly/new_issues.xlsx
+++ b/updates_weekly/new_issues.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -510,7 +510,7 @@
     <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="str">
         <f>_xll.BSRCH("FI:New Issues Brazil - EB2","cols=1;rows=25")</f>
-        <v>#N/A Requesting Data...</v>
+        <v>id</v>
       </c>
       <c r="F1" s="1"/>
     </row>

</xml_diff>